<commit_message>
task 63 final tuches
</commit_message>
<xml_diff>
--- a/metrics_column_report.xlsx
+++ b/metrics_column_report.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C44"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -455,7 +455,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1386</v>
+        <v>1385</v>
       </c>
     </row>
     <row r="3">
@@ -483,7 +483,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.917749</v>
+        <v>0.862094</v>
       </c>
     </row>
     <row r="5">
@@ -496,7 +496,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.936013</v>
+        <v>0.9048890000000001</v>
       </c>
     </row>
     <row r="6">
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.858155</v>
+        <v>0.837232</v>
       </c>
     </row>
     <row r="7">
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.885729</v>
+        <v>0.856332</v>
       </c>
     </row>
     <row r="8">
@@ -531,11 +531,11 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Precision_micro</t>
+          <t>AUC_ovr_multiclass</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.917749</v>
+        <v>0.423278</v>
       </c>
     </row>
     <row r="9">
@@ -544,11 +544,11 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Recall_micro</t>
+          <t>Brier_multiclass</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.917749</v>
+        <v>0.76561019</v>
       </c>
     </row>
     <row r="10">
@@ -557,11 +557,11 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>F1_micro</t>
+          <t>Brier_decomp_0_brier</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.917749</v>
+        <v>0.22373382</v>
       </c>
     </row>
     <row r="11">
@@ -570,11 +570,11 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>MCC</t>
+          <t>Brier_decomp_0_reliability</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.882283</v>
+        <v>0.17037382</v>
       </c>
     </row>
     <row r="12">
@@ -583,11 +583,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Class_0_Precision</t>
+          <t>Brier_decomp_0_resolution</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.920455</v>
+        <v>0.15821267</v>
       </c>
     </row>
     <row r="13">
@@ -596,11 +596,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Class_0_Recall</t>
+          <t>Brier_decomp_0_uncertainty</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.961995</v>
+        <v>0.21157268</v>
       </c>
     </row>
     <row r="14">
@@ -609,11 +609,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Class_0_F1</t>
+          <t>Brier_decomp_1_brier</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.940767</v>
+        <v>0.22620119</v>
       </c>
     </row>
     <row r="15">
@@ -622,11 +622,11 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Class_1_Precision</t>
+          <t>Brier_decomp_1_reliability</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.908705</v>
+        <v>0.05869063</v>
       </c>
     </row>
     <row r="16">
@@ -635,11 +635,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Class_1_Recall</t>
+          <t>Brier_decomp_1_resolution</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.91453</v>
+        <v>0.05598042</v>
       </c>
     </row>
     <row r="17">
@@ -648,11 +648,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Class_1_F1</t>
+          <t>Brier_decomp_1_uncertainty</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.911608</v>
+        <v>0.22349099</v>
       </c>
     </row>
     <row r="18">
@@ -661,11 +661,11 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Class_2_Precision</t>
+          <t>Brier_decomp_2_brier</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.914894</v>
+        <v>0.22187648</v>
       </c>
     </row>
     <row r="19">
@@ -674,11 +674,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Class_2_Recall</t>
+          <t>Brier_decomp_2_reliability</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.937046</v>
+        <v>0.14092458</v>
       </c>
     </row>
     <row r="20">
@@ -687,11 +687,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Class_2_F1</t>
+          <t>Brier_decomp_2_resolution</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.925837</v>
+        <v>0.12832282</v>
       </c>
     </row>
     <row r="21">
@@ -700,11 +700,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Class_3_Precision</t>
+          <t>Brier_decomp_2_uncertainty</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
+        <v>0.20927472</v>
       </c>
     </row>
     <row r="22">
@@ -713,11 +713,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Class_3_Recall</t>
+          <t>Brier_decomp_3_brier</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.619048</v>
+        <v>0.09379034</v>
       </c>
     </row>
     <row r="23">
@@ -726,11 +726,11 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Class_3_F1</t>
+          <t>Brier_decomp_3_reliability</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.764706</v>
+        <v>0.04225775</v>
       </c>
     </row>
     <row r="24">
@@ -739,13 +739,11 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ConfusionMatrix_shape</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>4x4</t>
-        </is>
+          <t>Brier_decomp_3_resolution</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>0.00543883</v>
       </c>
     </row>
     <row r="25">
@@ -754,260 +752,11 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CM[0,0]</t>
+          <t>Brier_decomp_3_uncertainty</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>405</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="n">
-        <v>25</v>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>CM[0,1]</t>
-        </is>
-      </c>
-      <c r="C26" t="n">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="n">
-        <v>26</v>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>CM[0,2]</t>
-        </is>
-      </c>
-      <c r="C27" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="n">
-        <v>27</v>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>CM[0,3]</t>
-        </is>
-      </c>
-      <c r="C28" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="n">
-        <v>28</v>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>CM[1,0]</t>
-        </is>
-      </c>
-      <c r="C29" t="n">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="n">
-        <v>29</v>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>CM[1,1]</t>
-        </is>
-      </c>
-      <c r="C30" t="n">
-        <v>428</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="n">
-        <v>30</v>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>CM[1,2]</t>
-        </is>
-      </c>
-      <c r="C31" t="n">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="n">
-        <v>31</v>
-      </c>
-      <c r="B32" t="inlineStr">
-        <is>
-          <t>CM[1,3]</t>
-        </is>
-      </c>
-      <c r="C32" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="n">
-        <v>32</v>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>CM[2,0]</t>
-        </is>
-      </c>
-      <c r="C33" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="n">
-        <v>33</v>
-      </c>
-      <c r="B34" t="inlineStr">
-        <is>
-          <t>CM[2,1]</t>
-        </is>
-      </c>
-      <c r="C34" t="n">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="n">
-        <v>34</v>
-      </c>
-      <c r="B35" t="inlineStr">
-        <is>
-          <t>CM[2,2]</t>
-        </is>
-      </c>
-      <c r="C35" t="n">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="n">
-        <v>35</v>
-      </c>
-      <c r="B36" t="inlineStr">
-        <is>
-          <t>CM[2,3]</t>
-        </is>
-      </c>
-      <c r="C36" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37">
-      <c r="A37" t="n">
-        <v>36</v>
-      </c>
-      <c r="B37" t="inlineStr">
-        <is>
-          <t>CM[3,0]</t>
-        </is>
-      </c>
-      <c r="C37" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" t="n">
-        <v>37</v>
-      </c>
-      <c r="B38" t="inlineStr">
-        <is>
-          <t>CM[3,1]</t>
-        </is>
-      </c>
-      <c r="C38" t="n">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="n">
-        <v>38</v>
-      </c>
-      <c r="B39" t="inlineStr">
-        <is>
-          <t>CM[3,2]</t>
-        </is>
-      </c>
-      <c r="C39" t="n">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="n">
-        <v>39</v>
-      </c>
-      <c r="B40" t="inlineStr">
-        <is>
-          <t>CM[3,3]</t>
-        </is>
-      </c>
-      <c r="C40" t="n">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="n">
-        <v>40</v>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>AUC_ovr_multiclass</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr"/>
-    </row>
-    <row r="42">
-      <c r="A42" t="n">
-        <v>41</v>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Brier_multiclass_error</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>index 3 is out of bounds for axis 1 with size 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>42</v>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Brier_decomp_error</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>index 3 is out of bounds for axis 1 with size 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
-        <v>43</v>
-      </c>
-      <c r="B44" t="inlineStr">
-        <is>
-          <t>Markedness</t>
-        </is>
-      </c>
-      <c r="C44" t="n">
-        <v>0.9081090000000001</v>
+        <v>0.05697142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update the code and start the task 65
</commit_message>
<xml_diff>
--- a/metrics_column_report.xlsx
+++ b/metrics_column_report.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -455,7 +455,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1385</v>
+        <v>1073</v>
       </c>
     </row>
     <row r="3">
@@ -469,7 +469,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0,1,2,3</t>
+          <t>0,1,2</t>
         </is>
       </c>
     </row>
@@ -483,7 +483,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.862094</v>
+        <v>0.848089</v>
       </c>
     </row>
     <row r="5">
@@ -496,7 +496,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>0.9048890000000001</v>
+        <v>0.76845</v>
       </c>
     </row>
     <row r="6">
@@ -509,7 +509,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.837232</v>
+        <v>0.540484</v>
       </c>
     </row>
     <row r="7">
@@ -522,7 +522,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.856332</v>
+        <v>0.59004</v>
       </c>
     </row>
     <row r="8">
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>0.423278</v>
+        <v>0.793341</v>
       </c>
     </row>
     <row r="9">
@@ -548,7 +548,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>0.76561019</v>
+        <v>0.2436069</v>
       </c>
     </row>
     <row r="10">
@@ -561,7 +561,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>0.22373382</v>
+        <v>0.1078015</v>
       </c>
     </row>
     <row r="11">
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>0.17037382</v>
+        <v>0.00047797</v>
       </c>
     </row>
     <row r="12">
@@ -587,7 +587,7 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>0.15821267</v>
+        <v>0.0573123</v>
       </c>
     </row>
     <row r="13">
@@ -600,7 +600,7 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>0.21157268</v>
+        <v>0.16463583</v>
       </c>
     </row>
     <row r="14">
@@ -613,7 +613,7 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0.22620119</v>
+        <v>0.06458406999999999</v>
       </c>
     </row>
     <row r="15">
@@ -626,7 +626,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.05869063</v>
+        <v>0.00030162</v>
       </c>
     </row>
     <row r="16">
@@ -639,7 +639,7 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.05598042</v>
+        <v>0.02098597</v>
       </c>
     </row>
     <row r="17">
@@ -652,7 +652,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.22349099</v>
+        <v>0.08526842</v>
       </c>
     </row>
     <row r="18">
@@ -665,7 +665,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.22187648</v>
+        <v>0.08488909</v>
       </c>
     </row>
     <row r="19">
@@ -678,7 +678,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.14092458</v>
+        <v>0.00027983</v>
       </c>
     </row>
     <row r="20">
@@ -691,7 +691,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.12832282</v>
+        <v>0.01616297</v>
       </c>
     </row>
     <row r="21">
@@ -704,59 +704,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.20927472</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="n">
-        <v>21</v>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>Brier_decomp_3_brier</t>
-        </is>
-      </c>
-      <c r="C22" t="n">
-        <v>0.09379034</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="n">
-        <v>22</v>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Brier_decomp_3_reliability</t>
-        </is>
-      </c>
-      <c r="C23" t="n">
-        <v>0.04225775</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="n">
-        <v>23</v>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Brier_decomp_3_resolution</t>
-        </is>
-      </c>
-      <c r="C24" t="n">
-        <v>0.00543883</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="n">
-        <v>24</v>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Brier_decomp_3_uncertainty</t>
-        </is>
-      </c>
-      <c r="C25" t="n">
-        <v>0.05697142</v>
+        <v>0.10077224</v>
       </c>
     </row>
   </sheetData>

</xml_diff>